<commit_message>
new schema for siswa dan nilai dan nilaiakhir
</commit_message>
<xml_diff>
--- a/public/down/Template_InputNilaiSiswa.xlsx
+++ b/public/down/Template_InputNilaiSiswa.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25330"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Indraaaa\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Indraa\Documents\codingan\SiNilai\public\down\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1C3DFB9A-8F14-45CD-8981-40E59C982720}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F12268C8-7F9E-424D-AF87-2D39D7EEB538}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" xr2:uid="{110F06B0-E56B-4C1E-AA87-941E3C259BC3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{110F06B0-E56B-4C1E-AA87-941E3C259BC3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>nis</t>
   </si>
@@ -46,13 +45,40 @@
     <t>kelas</t>
   </si>
   <si>
-    <t>value_daily</t>
-  </si>
-  <si>
-    <t>value_sts</t>
-  </si>
-  <si>
-    <t>value_sas</t>
+    <t>sumatif_2</t>
+  </si>
+  <si>
+    <t>sumatif_3</t>
+  </si>
+  <si>
+    <t>sumatif_4</t>
+  </si>
+  <si>
+    <t>sumatif_5</t>
+  </si>
+  <si>
+    <t>sumatif_6</t>
+  </si>
+  <si>
+    <t>sumatif_7</t>
+  </si>
+  <si>
+    <t>sumatif_8</t>
+  </si>
+  <si>
+    <t>sumatif_9</t>
+  </si>
+  <si>
+    <t>sumatif_10</t>
+  </si>
+  <si>
+    <t>sumatif_tengah</t>
+  </si>
+  <si>
+    <t>sumatif_akhir</t>
+  </si>
+  <si>
+    <t>sumatif_1</t>
   </si>
 </sst>
 </file>
@@ -404,10 +430,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB82F5B5-0880-4F69-AA42-76F5A412818A}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="11.5703125" customWidth="1"/>
+    <col min="5" max="8" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -418,13 +452,40 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>